<commit_message>
Add noncommercial PDFs and record upload decisions in evidence workbook
</commit_message>
<xml_diff>
--- a/evidence.xlsx
+++ b/evidence.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence table" sheetId="1" r:id="Rb48e0a7479e849d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding guide" sheetId="2" r:id="Rdabc95d87484462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence table" sheetId="1" r:id="R50c5e38f43624a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding guide" sheetId="2" r:id="R1bb4f0b7966b42ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -57,8 +57,12 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -78,6 +82,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFAFCFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -248,7 +257,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="64">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -425,17 +434,50 @@
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="1">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C2929"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceTable" displayName="EvidenceTable" ref="A1:Z122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:Z122"/>
-  <x:tableColumns count="26">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceTable" displayName="EvidenceTable" ref="A1:AD122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:AD122"/>
+  <x:tableColumns count="30">
     <x:tableColumn id="1" name="Citation"/>
     <x:tableColumn id="2" name="Epoxy system"/>
     <x:tableColumn id="3" name="Source of the data"/>
@@ -462,6 +504,10 @@
     <x:tableColumn id="24" name="Formal UQ"/>
     <x:tableColumn id="25" name="Public data"/>
     <x:tableColumn id="26" name="Public code"/>
+    <x:tableColumn id="27" name="Full-text access status"/>
+    <x:tableColumn id="28" name="Repository PDF status"/>
+    <x:tableColumn id="29" name="Repository PDF link"/>
+    <x:tableColumn id="30" name="PDF license / Upload note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -688,6 +734,10 @@
     <x:col min="24" max="24" width="12" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="12" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="12" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="25" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="34" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="53" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -769,6 +819,18 @@
       <x:c r="Z1" s="8" t="str">
         <x:v>Public code</x:v>
       </x:c>
+      <x:c r="AA1" s="70" t="str">
+        <x:v>Full-text access status</x:v>
+      </x:c>
+      <x:c r="AB1" s="70" t="str">
+        <x:v>Repository PDF status</x:v>
+      </x:c>
+      <x:c r="AC1" s="70" t="str">
+        <x:v>Repository PDF link</x:v>
+      </x:c>
+      <x:c r="AD1" s="70" t="str">
+        <x:v>PDF license / Upload note</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="9" t="str">
@@ -849,6 +911,18 @@
       <x:c r="Z2" s="18" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA2" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB2" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC2" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-001.pdf</x:v>
+      </x:c>
+      <x:c r="AD2" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
@@ -929,6 +1003,16 @@
       <x:c r="Z3" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA3" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB3" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC3" s="66"/>
+      <x:c r="AD3" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
@@ -1009,6 +1093,16 @@
       <x:c r="Z4" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA4" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB4" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC4" s="66"/>
+      <x:c r="AD4" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="str">
@@ -1089,6 +1183,16 @@
       <x:c r="Z5" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA5" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB5" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC5" s="66"/>
+      <x:c r="AD5" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="str">
@@ -1169,6 +1273,16 @@
       <x:c r="Z6" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA6" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB6" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC6" s="66"/>
+      <x:c r="AD6" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="str">
@@ -1249,6 +1363,18 @@
       <x:c r="Z7" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA7" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB7" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC7" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-006.pdf</x:v>
+      </x:c>
+      <x:c r="AD7" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="str">
@@ -1329,6 +1455,16 @@
       <x:c r="Z8" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA8" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB8" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC8" s="66"/>
+      <x:c r="AD8" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="str">
@@ -1409,6 +1545,18 @@
       <x:c r="Z9" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA9" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB9" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC9" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-008.pdf</x:v>
+      </x:c>
+      <x:c r="AD9" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
@@ -1489,6 +1637,16 @@
       <x:c r="Z10" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA10" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB10" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC10" s="66"/>
+      <x:c r="AD10" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
@@ -1569,6 +1727,16 @@
       <x:c r="Z11" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA11" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB11" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC11" s="66"/>
+      <x:c r="AD11" s="66" t="str">
+        <x:v>No article-specific redistribution license identified in the local PDF.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
@@ -1649,6 +1817,18 @@
       <x:c r="Z12" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA12" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB12" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC12" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-011.pdf</x:v>
+      </x:c>
+      <x:c r="AD12" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="10" t="str">
@@ -1729,6 +1909,16 @@
       <x:c r="Z13" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA13" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB13" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC13" s="66"/>
+      <x:c r="AD13" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="10" t="str">
@@ -1809,6 +1999,18 @@
       <x:c r="Z14" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA14" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB14" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC14" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-013.pdf</x:v>
+      </x:c>
+      <x:c r="AD14" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="10" t="str">
@@ -1889,6 +2091,16 @@
       <x:c r="Z15" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA15" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB15" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC15" s="66"/>
+      <x:c r="AD15" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="10" t="str">
@@ -1969,6 +2181,16 @@
       <x:c r="Z16" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA16" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB16" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC16" s="66"/>
+      <x:c r="AD16" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="10" t="str">
@@ -2049,6 +2271,18 @@
       <x:c r="Z17" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA17" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB17" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC17" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-016.pdf</x:v>
+      </x:c>
+      <x:c r="AD17" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="10" t="str">
@@ -2129,6 +2363,16 @@
       <x:c r="Z18" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA18" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB18" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC18" s="66"/>
+      <x:c r="AD18" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="10" t="str">
@@ -2209,6 +2453,18 @@
       <x:c r="Z19" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA19" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB19" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC19" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-018.pdf</x:v>
+      </x:c>
+      <x:c r="AD19" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="10" t="str">
@@ -2289,6 +2545,18 @@
       <x:c r="Z20" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA20" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB20" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC20" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-019.pdf</x:v>
+      </x:c>
+      <x:c r="AD20" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="10" t="str">
@@ -2369,6 +2637,16 @@
       <x:c r="Z21" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA21" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB21" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC21" s="66"/>
+      <x:c r="AD21" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="10" t="str">
@@ -2449,6 +2727,16 @@
       <x:c r="Z22" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA22" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB22" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC22" s="66"/>
+      <x:c r="AD22" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="10" t="str">
@@ -2529,6 +2817,16 @@
       <x:c r="Z23" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA23" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB23" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC23" s="66"/>
+      <x:c r="AD23" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="10" t="str">
@@ -2609,6 +2907,18 @@
       <x:c r="Z24" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA24" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB24" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC24" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-023.pdf</x:v>
+      </x:c>
+      <x:c r="AD24" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="10" t="str">
@@ -2689,6 +2999,16 @@
       <x:c r="Z25" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA25" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB25" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC25" s="66"/>
+      <x:c r="AD25" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="10" t="str">
@@ -2769,6 +3089,18 @@
       <x:c r="Z26" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA26" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB26" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC26" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-025.pdf</x:v>
+      </x:c>
+      <x:c r="AD26" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="10" t="str">
@@ -2849,6 +3181,16 @@
       <x:c r="Z27" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA27" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB27" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC27" s="66"/>
+      <x:c r="AD27" s="66" t="str">
+        <x:v>Conflicting license details: visible text says CC BY-NC; its link targets CC BY-NC-ND 4.0. Withheld pending clarification.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="10" t="str">
@@ -2929,6 +3271,18 @@
       <x:c r="Z28" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA28" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB28" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC28" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-027.pdf</x:v>
+      </x:c>
+      <x:c r="AD28" s="66" t="str">
+        <x:v>CC BY-SA 4.0. https://creativecommons.org/licenses/by-sa/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="10" t="str">
@@ -3009,6 +3363,18 @@
       <x:c r="Z29" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA29" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB29" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC29" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-028.pdf</x:v>
+      </x:c>
+      <x:c r="AD29" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="10" t="str">
@@ -3089,6 +3455,18 @@
       <x:c r="Z30" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA30" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB30" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC30" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-029.pdf</x:v>
+      </x:c>
+      <x:c r="AD30" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="10" t="str">
@@ -3169,6 +3547,16 @@
       <x:c r="Z31" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA31" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB31" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC31" s="66"/>
+      <x:c r="AD31" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="10" t="str">
@@ -3249,6 +3637,16 @@
       <x:c r="Z32" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA32" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB32" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC32" s="66"/>
+      <x:c r="AD32" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
@@ -3329,6 +3727,16 @@
       <x:c r="Z33" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA33" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB33" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC33" s="66"/>
+      <x:c r="AD33" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10" t="str">
@@ -3409,6 +3817,16 @@
       <x:c r="Z34" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA34" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB34" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC34" s="66"/>
+      <x:c r="AD34" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10" t="str">
@@ -3489,6 +3907,16 @@
       <x:c r="Z35" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA35" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB35" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC35" s="66"/>
+      <x:c r="AD35" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="10" t="str">
@@ -3569,6 +3997,16 @@
       <x:c r="Z36" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA36" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB36" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC36" s="66"/>
+      <x:c r="AD36" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10" t="str">
@@ -3649,6 +4087,16 @@
       <x:c r="Z37" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA37" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB37" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC37" s="66"/>
+      <x:c r="AD37" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="10" t="str">
@@ -3729,6 +4177,18 @@
       <x:c r="Z38" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA38" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB38" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC38" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-037.pdf</x:v>
+      </x:c>
+      <x:c r="AD38" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10" t="str">
@@ -3809,6 +4269,16 @@
       <x:c r="Z39" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA39" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB39" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC39" s="66"/>
+      <x:c r="AD39" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="10" t="str">
@@ -3889,6 +4359,18 @@
       <x:c r="Z40" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA40" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB40" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC40" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-039.pdf</x:v>
+      </x:c>
+      <x:c r="AD40" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10" t="str">
@@ -3969,6 +4451,18 @@
       <x:c r="Z41" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA41" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB41" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC41" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-040.pdf</x:v>
+      </x:c>
+      <x:c r="AD41" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="10" t="str">
@@ -4049,6 +4543,18 @@
       <x:c r="Z42" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA42" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB42" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC42" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-041.pdf</x:v>
+      </x:c>
+      <x:c r="AD42" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10" t="str">
@@ -4129,6 +4635,16 @@
       <x:c r="Z43" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA43" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB43" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC43" s="66"/>
+      <x:c r="AD43" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="10" t="str">
@@ -4209,6 +4725,16 @@
       <x:c r="Z44" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA44" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB44" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC44" s="66"/>
+      <x:c r="AD44" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="10" t="str">
@@ -4289,6 +4815,16 @@
       <x:c r="Z45" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA45" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB45" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC45" s="66"/>
+      <x:c r="AD45" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="10" t="str">
@@ -4369,6 +4905,16 @@
       <x:c r="Z46" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA46" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB46" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC46" s="66"/>
+      <x:c r="AD46" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="10" t="str">
@@ -4449,6 +4995,18 @@
       <x:c r="Z47" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA47" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB47" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC47" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-046.pdf</x:v>
+      </x:c>
+      <x:c r="AD47" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="10" t="str">
@@ -4529,6 +5087,16 @@
       <x:c r="Z48" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA48" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB48" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC48" s="66"/>
+      <x:c r="AD48" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="10" t="str">
@@ -4609,6 +5177,18 @@
       <x:c r="Z49" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA49" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB49" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC49" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-048.pdf</x:v>
+      </x:c>
+      <x:c r="AD49" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="10" t="str">
@@ -4689,6 +5269,18 @@
       <x:c r="Z50" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA50" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB50" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC50" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-049.pdf</x:v>
+      </x:c>
+      <x:c r="AD50" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="10" t="str">
@@ -4769,6 +5361,18 @@
       <x:c r="Z51" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA51" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB51" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC51" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-050.pdf</x:v>
+      </x:c>
+      <x:c r="AD51" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="10" t="str">
@@ -4849,6 +5453,16 @@
       <x:c r="Z52" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA52" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB52" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC52" s="66"/>
+      <x:c r="AD52" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="10" t="str">
@@ -4929,6 +5543,18 @@
       <x:c r="Z53" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA53" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB53" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC53" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-052.pdf</x:v>
+      </x:c>
+      <x:c r="AD53" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="10" t="str">
@@ -5009,6 +5635,18 @@
       <x:c r="Z54" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA54" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB54" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC54" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-053.pdf</x:v>
+      </x:c>
+      <x:c r="AD54" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="10" t="str">
@@ -5089,6 +5727,16 @@
       <x:c r="Z55" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA55" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB55" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC55" s="66"/>
+      <x:c r="AD55" s="66" t="str">
+        <x:v>The source table links a repository copy; redistribution permission for this local publisher PDF was not established.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="10" t="str">
@@ -5169,6 +5817,16 @@
       <x:c r="Z56" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA56" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB56" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC56" s="66"/>
+      <x:c r="AD56" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="10" t="str">
@@ -5249,6 +5907,16 @@
       <x:c r="Z57" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA57" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB57" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC57" s="66"/>
+      <x:c r="AD57" s="66" t="str">
+        <x:v>No article-specific redistribution license identified in the local conference manuscript.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="10" t="str">
@@ -5329,6 +5997,18 @@
       <x:c r="Z58" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA58" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB58" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC58" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-057.pdf</x:v>
+      </x:c>
+      <x:c r="AD58" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="10" t="str">
@@ -5409,6 +6089,16 @@
       <x:c r="Z59" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA59" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB59" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC59" s="66"/>
+      <x:c r="AD59" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="10" t="str">
@@ -5489,6 +6179,18 @@
       <x:c r="Z60" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA60" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB60" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC60" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-059.pdf</x:v>
+      </x:c>
+      <x:c r="AD60" s="66" t="str">
+        <x:v>CC BY-NC 4.0. https://creativecommons.org/licenses/by-nc/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="10" t="str">
@@ -5569,6 +6271,16 @@
       <x:c r="Z61" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA61" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB61" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC61" s="66"/>
+      <x:c r="AD61" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="10" t="str">
@@ -5649,6 +6361,16 @@
       <x:c r="Z62" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA62" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB62" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC62" s="66"/>
+      <x:c r="AD62" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="10" t="str">
@@ -5729,6 +6451,16 @@
       <x:c r="Z63" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA63" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB63" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC63" s="66"/>
+      <x:c r="AD63" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="10" t="str">
@@ -5809,6 +6541,16 @@
       <x:c r="Z64" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA64" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB64" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC64" s="66"/>
+      <x:c r="AD64" s="66" t="str">
+        <x:v>Generic Wiley footer is not an article-specific open license; source table reports bronze OA.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="10" t="str">
@@ -5889,6 +6631,18 @@
       <x:c r="Z65" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA65" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB65" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC65" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-064.pdf</x:v>
+      </x:c>
+      <x:c r="AD65" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="10" t="str">
@@ -5969,6 +6723,16 @@
       <x:c r="Z66" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA66" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB66" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC66" s="66"/>
+      <x:c r="AD66" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="10" t="str">
@@ -6049,6 +6813,16 @@
       <x:c r="Z67" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA67" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB67" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC67" s="66"/>
+      <x:c r="AD67" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="10" t="str">
@@ -6129,6 +6903,18 @@
       <x:c r="Z68" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA68" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB68" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC68" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-067.pdf</x:v>
+      </x:c>
+      <x:c r="AD68" s="66" t="str">
+        <x:v>CC BY-NC 4.0. https://creativecommons.org/licenses/by-nc/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="10" t="str">
@@ -6209,6 +6995,16 @@
       <x:c r="Z69" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA69" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB69" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC69" s="66"/>
+      <x:c r="AD69" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="10" t="str">
@@ -6289,6 +7085,18 @@
       <x:c r="Z70" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA70" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB70" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC70" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-069.pdf</x:v>
+      </x:c>
+      <x:c r="AD70" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="10" t="str">
@@ -6369,6 +7177,16 @@
       <x:c r="Z71" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA71" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB71" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC71" s="66"/>
+      <x:c r="AD71" s="66" t="str">
+        <x:v>No article-specific redistribution license identified; source table reports bronze OA.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="10" t="str">
@@ -6449,6 +7267,16 @@
       <x:c r="Z72" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA72" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB72" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC72" s="66"/>
+      <x:c r="AD72" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="10" t="str">
@@ -6529,6 +7357,16 @@
       <x:c r="Z73" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA73" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB73" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC73" s="66"/>
+      <x:c r="AD73" s="66" t="str">
+        <x:v>No article-specific redistribution license identified in the local PDF.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="10" t="str">
@@ -6609,6 +7447,16 @@
       <x:c r="Z74" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA74" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB74" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC74" s="66"/>
+      <x:c r="AD74" s="66" t="str">
+        <x:v>No article-specific redistribution license identified; source access metadata is conflicting.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="10" t="str">
@@ -6689,6 +7537,16 @@
       <x:c r="Z75" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA75" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB75" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC75" s="66"/>
+      <x:c r="AD75" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="10" t="str">
@@ -6769,6 +7627,18 @@
       <x:c r="Z76" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA76" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB76" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC76" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-075.pdf</x:v>
+      </x:c>
+      <x:c r="AD76" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="10" t="str">
@@ -6849,6 +7719,16 @@
       <x:c r="Z77" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA77" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB77" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC77" s="66"/>
+      <x:c r="AD77" s="66" t="str">
+        <x:v>Generic Wiley footer is not an article-specific open license; source table reports bronze OA.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="10" t="str">
@@ -6929,6 +7809,16 @@
       <x:c r="Z78" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA78" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB78" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC78" s="66"/>
+      <x:c r="AD78" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="10" t="str">
@@ -7009,6 +7899,16 @@
       <x:c r="Z79" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA79" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB79" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC79" s="66"/>
+      <x:c r="AD79" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="10" t="str">
@@ -7089,6 +7989,18 @@
       <x:c r="Z80" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA80" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB80" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC80" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-079.pdf</x:v>
+      </x:c>
+      <x:c r="AD80" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="10" t="str">
@@ -7169,6 +8081,18 @@
       <x:c r="Z81" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA81" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB81" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC81" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-080.pdf</x:v>
+      </x:c>
+      <x:c r="AD81" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="10" t="str">
@@ -7249,6 +8173,16 @@
       <x:c r="Z82" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA82" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB82" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC82" s="66"/>
+      <x:c r="AD82" s="66" t="str">
+        <x:v>Local publisher PDF states All rights reserved; the source table links a different preprint version.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="10" t="str">
@@ -7329,6 +8263,16 @@
       <x:c r="Z83" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA83" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB83" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC83" s="66"/>
+      <x:c r="AD83" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="10" t="str">
@@ -7409,6 +8353,16 @@
       <x:c r="Z84" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA84" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB84" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC84" s="66"/>
+      <x:c r="AD84" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="10" t="str">
@@ -7489,6 +8443,16 @@
       <x:c r="Z85" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA85" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB85" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC85" s="66"/>
+      <x:c r="AD85" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="10" t="str">
@@ -7569,6 +8533,16 @@
       <x:c r="Z86" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA86" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB86" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC86" s="66"/>
+      <x:c r="AD86" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="10" t="str">
@@ -7649,6 +8623,18 @@
       <x:c r="Z87" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA87" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB87" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC87" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-086.pdf</x:v>
+      </x:c>
+      <x:c r="AD87" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="10" t="str">
@@ -7729,6 +8715,16 @@
       <x:c r="Z88" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA88" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB88" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC88" s="66"/>
+      <x:c r="AD88" s="66" t="str">
+        <x:v>Local file contains personal markup annotations; a clean publisher version is required before sharing under CC BY-NC-ND.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="10" t="str">
@@ -7809,6 +8805,16 @@
       <x:c r="Z89" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA89" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB89" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC89" s="66"/>
+      <x:c r="AD89" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="10" t="str">
@@ -7889,6 +8895,16 @@
       <x:c r="Z90" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA90" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB90" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC90" s="66"/>
+      <x:c r="AD90" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="10" t="str">
@@ -7969,6 +8985,16 @@
       <x:c r="Z91" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA91" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB91" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC91" s="66"/>
+      <x:c r="AD91" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="10" t="str">
@@ -8049,6 +9075,16 @@
       <x:c r="Z92" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA92" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB92" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC92" s="66"/>
+      <x:c r="AD92" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="10" t="str">
@@ -8129,6 +9165,16 @@
       <x:c r="Z93" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA93" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB93" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC93" s="66"/>
+      <x:c r="AD93" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="10" t="str">
@@ -8209,6 +9255,16 @@
       <x:c r="Z94" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA94" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB94" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC94" s="66"/>
+      <x:c r="AD94" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="10" t="str">
@@ -8289,6 +9345,16 @@
       <x:c r="Z95" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA95" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB95" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC95" s="66"/>
+      <x:c r="AD95" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="10" t="str">
@@ -8369,6 +9435,16 @@
       <x:c r="Z96" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA96" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB96" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC96" s="66"/>
+      <x:c r="AD96" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="10" t="str">
@@ -8449,6 +9525,18 @@
       <x:c r="Z97" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA97" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB97" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC97" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-096.pdf</x:v>
+      </x:c>
+      <x:c r="AD97" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="10" t="str">
@@ -8529,6 +9617,16 @@
       <x:c r="Z98" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA98" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB98" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC98" s="66"/>
+      <x:c r="AD98" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="10" t="str">
@@ -8609,6 +9707,16 @@
       <x:c r="Z99" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA99" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB99" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC99" s="66"/>
+      <x:c r="AD99" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="10" t="str">
@@ -8689,6 +9797,16 @@
       <x:c r="Z100" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA100" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB100" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC100" s="66"/>
+      <x:c r="AD100" s="66" t="str">
+        <x:v>Generic Wiley footer is not an article-specific open license; source table reports bronze OA.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="10" t="str">
@@ -8769,6 +9887,16 @@
       <x:c r="Z101" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA101" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB101" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC101" s="66"/>
+      <x:c r="AD101" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="10" t="str">
@@ -8849,6 +9977,16 @@
       <x:c r="Z102" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA102" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB102" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC102" s="66"/>
+      <x:c r="AD102" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="10" t="str">
@@ -8929,6 +10067,16 @@
       <x:c r="Z103" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA103" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB103" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC103" s="66"/>
+      <x:c r="AD103" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="10" t="str">
@@ -9009,6 +10157,18 @@
       <x:c r="Z104" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA104" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB104" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC104" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-103.pdf</x:v>
+      </x:c>
+      <x:c r="AD104" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="10" t="str">
@@ -9089,6 +10249,16 @@
       <x:c r="Z105" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA105" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB105" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC105" s="66"/>
+      <x:c r="AD105" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="10" t="str">
@@ -9169,6 +10339,18 @@
       <x:c r="Z106" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA106" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB106" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC106" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-105.pdf</x:v>
+      </x:c>
+      <x:c r="AD106" s="66" t="str">
+        <x:v>CC BY-NC-ND 4.0. https://creativecommons.org/licenses/by-nc-nd/4.0/ Unmodified copy; retain attribution and notices. Noncommercial use only. Do not distribute adaptations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="10" t="str">
@@ -9249,6 +10431,16 @@
       <x:c r="Z107" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA107" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB107" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC107" s="66"/>
+      <x:c r="AD107" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="10" t="str">
@@ -9329,6 +10521,18 @@
       <x:c r="Z108" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA108" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB108" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC108" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-107.pdf</x:v>
+      </x:c>
+      <x:c r="AD108" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="10" t="str">
@@ -9409,6 +10613,16 @@
       <x:c r="Z109" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA109" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB109" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC109" s="66"/>
+      <x:c r="AD109" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="10" t="str">
@@ -9489,6 +10703,18 @@
       <x:c r="Z110" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA110" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB110" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC110" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-109.pdf</x:v>
+      </x:c>
+      <x:c r="AD110" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="10" t="str">
@@ -9569,6 +10795,18 @@
       <x:c r="Z111" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA111" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB111" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC111" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-110.pdf</x:v>
+      </x:c>
+      <x:c r="AD111" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="10" t="str">
@@ -9649,6 +10887,18 @@
       <x:c r="Z112" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA112" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB112" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC112" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-111.pdf</x:v>
+      </x:c>
+      <x:c r="AD112" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="10" t="str">
@@ -9729,6 +10979,16 @@
       <x:c r="Z113" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA113" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB113" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC113" s="66"/>
+      <x:c r="AD113" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="10" t="str">
@@ -9809,6 +11069,18 @@
       <x:c r="Z114" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA114" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB114" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC114" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-113.pdf</x:v>
+      </x:c>
+      <x:c r="AD114" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="10" t="str">
@@ -9889,6 +11161,18 @@
       <x:c r="Z115" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
+      <x:c r="AA115" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB115" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC115" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-114.pdf</x:v>
+      </x:c>
+      <x:c r="AD115" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="10" t="str">
@@ -9969,6 +11253,16 @@
       <x:c r="Z116" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA116" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB116" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC116" s="66"/>
+      <x:c r="AD116" s="66" t="str">
+        <x:v>Repository reading access does not establish permission to redistribute this local publisher PDF.</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="10" t="str">
@@ -10049,6 +11343,16 @@
       <x:c r="Z117" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA117" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB117" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC117" s="66"/>
+      <x:c r="AD117" s="66" t="str">
+        <x:v>Local file contains personal markup annotations; withheld to avoid publishing private annotation metadata.</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="10" t="str">
@@ -10129,6 +11433,16 @@
       <x:c r="Z118" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA118" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB118" s="66" t="str">
+        <x:v>Not uploaded - review required</x:v>
+      </x:c>
+      <x:c r="AC118" s="66"/>
+      <x:c r="AD118" s="66" t="str">
+        <x:v>Local file contains personal markup annotations; withheld to avoid publishing private annotation metadata.</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="10" t="str">
@@ -10209,6 +11523,16 @@
       <x:c r="Z119" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA119" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB119" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC119" s="66"/>
+      <x:c r="AD119" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="10" t="str">
@@ -10289,6 +11613,16 @@
       <x:c r="Z120" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA120" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB120" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC120" s="66"/>
+      <x:c r="AD120" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="10" t="str">
@@ -10369,6 +11703,16 @@
       <x:c r="Z121" s="19" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA121" s="66" t="str">
+        <x:v>Not publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB121" s="66" t="str">
+        <x:v>Not uploaded - public access unconfirmed</x:v>
+      </x:c>
+      <x:c r="AC121" s="66"/>
+      <x:c r="AD121" s="66" t="str">
+        <x:v>Source access table does not confirm public access; local PDF not reviewed for redistribution.</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="11" t="str">
@@ -10449,8 +11793,23 @@
       <x:c r="Z122" s="20" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="AA122" s="66" t="str">
+        <x:v>Publicly accessible</x:v>
+      </x:c>
+      <x:c r="AB122" s="66" t="str">
+        <x:v>Uploaded</x:v>
+      </x:c>
+      <x:c r="AC122" s="66" t="str">
+        <x:v>https://github.com/JingSu0627/epoxy-ml-evidence-map/blob/main/public_pdfs/EML-121.pdf</x:v>
+      </x:c>
+      <x:c r="AD122" s="66" t="str">
+        <x:v>CC BY 4.0. https://creativecommons.org/licenses/by/4.0/ Unmodified copy; retain attribution and notices.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="AB2:AB122">
+    <x:cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="Not uploaded"/>
+  </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="U2:Z122">
       <x:formula1>"Yes,No,Unclear,NA"</x:formula1>
@@ -10458,7 +11817,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0620a6e00ee4749"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R013a1c0d63624888"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>